<commit_message>
Revise template label print
</commit_message>
<xml_diff>
--- a/bin/Debug/Template/LabelSemiPrintTemplate.xlsx
+++ b/bin/Debug/Template/LabelSemiPrintTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project\MC-Dept-App\bin\Debug\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47AA1DEA-0AD1-4280-A2A1-3E295C158F97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8BF7216-449F-41AF-AFA1-8DA273B0827E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A6BDC683-4EB3-4F0D-B7D4-F6C0E6AB9432}"/>
   </bookViews>
@@ -33,27 +33,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
-  <si>
-    <t>លេខកូតរបស់WIP
-( WIP barcode )</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>Sub MT</t>
   </si>
   <si>
-    <t>OP MC</t>
-  </si>
-  <si>
     <t>MT OP</t>
   </si>
   <si>
     <t>☐ ថ្ងៃ   ☐ ​យប់</t>
   </si>
   <si>
-    <t xml:space="preserve"> ពណ៍នាពីការប្រើប្រាស់របស់ពិសេស[ Special Accept (S.A)Detall ]</t>
-  </si>
-  <si>
     <t xml:space="preserve"> កាលបរិច្ឆេទត្រួតពិនិត្យ(Inspect date)</t>
   </si>
   <si>
@@ -63,18 +53,9 @@
     <t xml:space="preserve"> ☐ OK   ☐ NG   ☐ ប្រើប្រាស់ជាពិសេស</t>
   </si>
   <si>
-    <t xml:space="preserve"> ក្រដាសបង្ហាញផលិតផល​ ​Product Label</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> REF:MC-RE-027 REV:01  Date:2020-11-16</t>
-  </si>
-  <si>
     <t xml:space="preserve"> ម៉ារ៉ូនិក(ខេមបូឌា) Marunix Cambodia</t>
   </si>
   <si>
-    <t xml:space="preserve"> ថ្ងៃចេញទំនេញ(D.Date)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> អ្នកប្រតិបត្តិម៉ាស៊ីន(Oparetor)</t>
   </si>
   <si>
@@ -84,9 +65,6 @@
     <t xml:space="preserve"> កំឡុងពេល(Shift)</t>
   </si>
   <si>
-    <t xml:space="preserve"> ថ្ងៃផលិត(Pro.date)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> ចំនួន១បាច់(Batch/ Qty)</t>
   </si>
   <si>
@@ -109,13 +87,38 @@
   </si>
   <si>
     <t xml:space="preserve"> ឈ្មោះផលិតផល</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> អ្នកត្រួតពិនិត្យ MQC</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ថ្ងៃផលិត(Pro.date) Auto</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ថ្ងៃផលិត(Pro.date) Semi</t>
+  </si>
+  <si>
+    <t>MC Leader</t>
+  </si>
+  <si>
+    <t>Semi No.</t>
+  </si>
+  <si>
+    <t>Semi PIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   ថ្ងៃចេញទំនេញ(D.Date)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   លេខកូតរបស់WIP
+    ( WIP barcode )</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,6 +164,12 @@
       <color theme="1"/>
       <name val="Khmer OS System"/>
     </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Khmer OS System"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -182,7 +191,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -264,6 +273,70 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -273,7 +346,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1">
       <alignment vertical="center"/>
@@ -281,83 +354,149 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -689,281 +828,321 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504C567F-7FC1-4C34-A445-146B619C93CE}">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="10" style="1" customWidth="1"/>
-    <col min="3" max="3" width="6.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="5.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="4.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="4.85546875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="11.85546875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="5" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="1"/>
+    <col min="3" max="4" width="5" style="1" customWidth="1"/>
+    <col min="5" max="6" width="5.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="4.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="3.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="4.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="5" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-    </row>
-    <row r="3" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="7"/>
+    <row r="1" spans="1:11" ht="18" customHeight="1" thickBot="1">
+      <c r="A1" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+    </row>
+    <row r="2" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
+      <c r="A2" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+    </row>
+    <row r="3" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
+      <c r="A3" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="22"/>
       <c r="C3" s="23"/>
       <c r="D3" s="24"/>
-      <c r="E3" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A4" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="7"/>
+      <c r="E3" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="12"/>
+    </row>
+    <row r="4" spans="1:11" ht="18" customHeight="1" thickBot="1">
+      <c r="A4" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="22"/>
       <c r="C4" s="23"/>
       <c r="D4" s="24"/>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="12"/>
+    </row>
+    <row r="5" spans="1:11" ht="18" customHeight="1" thickBot="1">
+      <c r="A5" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="22"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="12"/>
+    </row>
+    <row r="6" spans="1:11" ht="18" customHeight="1" thickBot="1">
+      <c r="A6" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="22"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="34" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="12"/>
+    </row>
+    <row r="7" spans="1:11" ht="18" customHeight="1" thickBot="1">
+      <c r="A7" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="22"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="12"/>
+    </row>
+    <row r="8" spans="1:11" ht="18" customHeight="1" thickBot="1">
+      <c r="A8" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="22"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="12"/>
+    </row>
+    <row r="9" spans="1:11" ht="18" customHeight="1" thickBot="1">
+      <c r="A9" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+    </row>
+    <row r="10" spans="1:11" ht="19.5" customHeight="1" thickBot="1">
+      <c r="A10" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="27"/>
+      <c r="C10" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" s="12"/>
+      <c r="E10" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10" s="14"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="49"/>
+    </row>
+    <row r="11" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
+      <c r="A11" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="25"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F11" s="8"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="50"/>
+    </row>
+    <row r="12" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
+      <c r="A12" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A5" s="7" t="s">
+      <c r="B12" s="25"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="20"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="21"/>
+    </row>
+    <row r="13" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
+      <c r="A13" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="14" t="s">
+      <c r="B13" s="25"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G13" s="10"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K13" s="2"/>
+    </row>
+    <row r="14" spans="1:11" ht="18" customHeight="1" thickBot="1">
+      <c r="A14" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A7" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A8" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="3"/>
-    </row>
-    <row r="9" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A9" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-    </row>
-    <row r="10" spans="1:9" ht="20.25" customHeight="1" thickBot="1">
-      <c r="A10" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" s="20"/>
-      <c r="E10" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
-    </row>
-    <row r="11" spans="1:9" ht="20.25" customHeight="1" thickBot="1">
-      <c r="A11" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-    </row>
-    <row r="12" spans="1:9" ht="28.5" customHeight="1" thickBot="1">
-      <c r="A12" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="F12" s="19"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:9" ht="20.25" customHeight="1" thickBot="1">
-      <c r="A13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="F13" s="21"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="1:9" ht="18" customHeight="1" thickBot="1">
-      <c r="A14" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-    </row>
-    <row r="15" spans="1:9" ht="19.5" customHeight="1" thickBot="1">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="25"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" s="36"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="45"/>
+      <c r="K14" s="46"/>
+    </row>
+    <row r="15" spans="1:11" ht="18.75" customHeight="1" thickBot="1">
+      <c r="A15" s="25"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="47"/>
+      <c r="K15" s="48"/>
     </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="47">
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
     <mergeCell ref="A14:D15"/>
-    <mergeCell ref="E14:I14"/>
-    <mergeCell ref="E15:I15"/>
+    <mergeCell ref="E14:G15"/>
+    <mergeCell ref="C13:E13"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="E10:I11"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
     <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:K9"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:I7"/>
+    <mergeCell ref="E8:I8"/>
+    <mergeCell ref="J8:K8"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:D8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:I9"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:H5"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:I2"/>
+    <mergeCell ref="C1:K2"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="H14:K15"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="H10:J11"/>
+    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.01" footer="0"/>
   <pageSetup paperSize="70" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix bug in budget
</commit_message>
<xml_diff>
--- a/bin/Debug/Template/LabelSemiPrintTemplate.xlsx
+++ b/bin/Debug/Template/LabelSemiPrintTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project\MC-Dept-App\bin\Debug\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60DDAA16-9BD9-476E-AF6B-7679C7A926E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11A9383-2250-414D-AD28-56ADBC69DE23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A6BDC683-4EB3-4F0D-B7D4-F6C0E6AB9432}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>Sub MT</t>
   </si>
@@ -112,6 +112,15 @@
   <si>
     <t xml:space="preserve">   លេខកូតរបស់WIP
     ( WIP barcode )</t>
+  </si>
+  <si>
+    <t>Total PCS</t>
+  </si>
+  <si>
+    <t>Qty / Box</t>
+  </si>
+  <si>
+    <t>Label No.</t>
   </si>
 </sst>
 </file>
@@ -171,7 +180,7 @@
       <name val="Khmer OS Siemreap"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -190,6 +199,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -346,7 +361,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1">
       <alignment vertical="center"/>
@@ -363,9 +378,108 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -393,109 +507,16 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="2" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="2" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -519,12 +540,26 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Memo"/>
       <sheetName val="Sheet1"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
+      <sheetData sheetId="0">
+        <row r="2">
+          <cell r="J2" t="str">
+            <v>SK-A20 (A)</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="J3" t="str">
+            <v>SK-A20 (B)</v>
+          </cell>
+        </row>
+      </sheetData>
       <sheetData sheetId="1"/>
     </sheetDataSet>
   </externalBook>
@@ -844,285 +879,275 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
     </row>
     <row r="2" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
     </row>
     <row r="3" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="28"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
       <c r="D3" s="30"/>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="19"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="16"/>
     </row>
     <row r="4" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="28"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="29"/>
       <c r="D4" s="30"/>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="19"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="16"/>
     </row>
     <row r="5" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="16" t="s">
+      <c r="B5" s="28"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="19"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="35"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="16"/>
     </row>
     <row r="6" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="25" t="s">
+      <c r="B6" s="28"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="19"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="16"/>
     </row>
     <row r="7" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="21"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="6" t="s">
+      <c r="B7" s="28"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="19"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="16"/>
     </row>
     <row r="8" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="21"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="16" t="s">
+      <c r="B8" s="28"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="19"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="16"/>
     </row>
     <row r="9" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="21"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="52"/>
+      <c r="E9" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="14"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="16"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="16"/>
     </row>
     <row r="10" spans="1:11" ht="19.5" customHeight="1" thickBot="1">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="18" t="s">
+      <c r="B10" s="33"/>
+      <c r="C10" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="19"/>
+      <c r="D10" s="16"/>
       <c r="E10" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="F10" s="34"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="38" t="s">
+      <c r="F10" s="10"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="I10" s="39"/>
-      <c r="J10" s="40"/>
-      <c r="K10" s="48"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="26"/>
     </row>
     <row r="11" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
+      <c r="B11" s="31"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
       <c r="E11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="F11" s="36"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="43"/>
-      <c r="K11" s="49"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="27"/>
     </row>
     <row r="12" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="31" t="s">
+      <c r="B12" s="31"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="32"/>
-      <c r="H12" s="31"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="33"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="25"/>
     </row>
     <row r="13" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="15"/>
+      <c r="B13" s="31"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="48"/>
       <c r="F13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="18"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="19"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="16"/>
       <c r="J13" s="2" t="s">
         <v>22</v>
       </c>
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="7" t="s">
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44"/>
-      <c r="K14" s="45"/>
+      <c r="F14" s="41"/>
+      <c r="G14" s="42"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="7"/>
     </row>
     <row r="15" spans="1:11" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="46"/>
-      <c r="K15" s="47"/>
+      <c r="A15" s="31"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="43"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="45"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="47">
-    <mergeCell ref="H14:K15"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="H10:J11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="K10:K11"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:I4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:K2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="J3:K3"/>
+  <mergeCells count="50">
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:D15"/>
+    <mergeCell ref="E14:G15"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C12:E12"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:K9"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="E6:I6"/>
@@ -1133,16 +1158,35 @@
     <mergeCell ref="J8:K8"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C8:D8"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:D15"/>
-    <mergeCell ref="E14:G15"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:K2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H14:K15"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="H10:J11"/>
+    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.01" footer="0"/>
   <pageSetup paperSize="70" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Finished master and revise semi label print
</commit_message>
<xml_diff>
--- a/bin/Debug/Template/LabelSemiPrintTemplate.xlsx
+++ b/bin/Debug/Template/LabelSemiPrintTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project\MC-Dept-App\bin\Debug\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98870E4-3225-4973-B306-6AAF6774B9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A20086E-AED1-4705-BAD7-4BFF8827FCEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A6BDC683-4EB3-4F0D-B7D4-F6C0E6AB9432}"/>
   </bookViews>
@@ -186,7 +186,7 @@
       <name val="Khmer OS System"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -205,12 +205,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -367,7 +361,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1">
       <alignment vertical="center"/>
@@ -387,6 +381,102 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="12" fontId="8" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="12" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="6" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -411,15 +501,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -437,99 +518,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="12" fontId="8" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="12" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -891,264 +879,304 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
     </row>
     <row r="2" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="37"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
     </row>
     <row r="3" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="32" t="s">
+      <c r="B3" s="22"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="17"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="20"/>
     </row>
     <row r="4" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="32" t="s">
+      <c r="B4" s="22"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="17"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="20"/>
     </row>
     <row r="5" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="29"/>
+      <c r="B5" s="22"/>
       <c r="C5" s="33"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="34" t="s">
+      <c r="D5" s="19"/>
+      <c r="E5" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="35"/>
-      <c r="G5" s="35"/>
-      <c r="H5" s="35"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="17"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="20"/>
     </row>
     <row r="6" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="29"/>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="42" t="s">
+      <c r="B6" s="22"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="42"/>
-      <c r="H6" s="42"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="17"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="20"/>
     </row>
     <row r="7" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="29"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="32" t="s">
+      <c r="B7" s="22"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="17"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="20"/>
     </row>
     <row r="8" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="34" t="s">
+      <c r="B8" s="22"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="17"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="20"/>
     </row>
     <row r="9" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="29"/>
-      <c r="C9" s="40" t="s">
+      <c r="B9" s="22"/>
+      <c r="C9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="41"/>
+      <c r="D9" s="16"/>
       <c r="E9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="15"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="15" t="s">
+      <c r="F9" s="19"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="I9" s="17"/>
-      <c r="J9" s="53"/>
-      <c r="K9" s="54"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="27"/>
     </row>
     <row r="10" spans="1:11" ht="19.5" customHeight="1" thickBot="1">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="15" t="s">
+      <c r="B10" s="17"/>
+      <c r="C10" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="17"/>
+      <c r="D10" s="20"/>
       <c r="E10" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="F10" s="11"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="18" t="s">
+      <c r="F10" s="43"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="I10" s="19"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="27"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="37"/>
     </row>
     <row r="11" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="52"/>
-      <c r="D11" s="52"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="23"/>
-      <c r="K11" s="28"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="50"/>
+      <c r="I11" s="51"/>
+      <c r="J11" s="52"/>
+      <c r="K11" s="38"/>
     </row>
     <row r="12" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="24" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="25"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="26"/>
+      <c r="G12" s="35"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="35"/>
+      <c r="J12" s="35"/>
+      <c r="K12" s="36"/>
     </row>
     <row r="13" spans="1:11" ht="17.25" customHeight="1" thickBot="1">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="50"/>
-      <c r="E13" s="51"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="16"/>
       <c r="F13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="15"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="17"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="20"/>
       <c r="J13" s="2" t="s">
         <v>22</v>
       </c>
       <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:11" ht="18" customHeight="1" thickBot="1">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="43" t="s">
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F14" s="44"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="8"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="39"/>
+      <c r="I14" s="39"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="40"/>
     </row>
     <row r="15" spans="1:11" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A15" s="32"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="46"/>
-      <c r="F15" s="47"/>
-      <c r="G15" s="48"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="10"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="41"/>
+      <c r="I15" s="41"/>
+      <c r="J15" s="41"/>
+      <c r="K15" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="50">
+    <mergeCell ref="H14:K15"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="H10:J11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:K2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="E8:I8"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:I7"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:D15"/>
     <mergeCell ref="E14:G15"/>
@@ -1159,46 +1187,6 @@
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C12:E12"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:I7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="E8:I8"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:K2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:I4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="K10:K11"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="H14:K15"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="H10:J11"/>
-    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.01" footer="0"/>
   <pageSetup paperSize="70" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>